<commit_message>
Fix role template coverage and placeholder XLSX artifacts
Regenerate all published role checklists, enforce XLSX integrity checks in both template directories, and align v1.8.0 release/version wording.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: d6ed2a9a-75d8-4330-bfd0-804c1778bf8b
</commit_message>
<xml_diff>
--- a/assessment/templates/compliance-officer-checklist.xlsx
+++ b/assessment/templates/compliance-officer-checklist.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compliance Officer'!$A$4:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compliance Officer'!$A$4:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: Compliance Officer  |  FSI Copilot Governance Framework v1.8  |  18 controls</t>
+          <t>Role: Compliance Officer  |  FSI Copilot Governance Framework v1.8.0  |  22 controls</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>3.8a</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>AI Disclosure, Transparency, and SEC Marketing Rule</t>
+          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Is AI disclosure language presented to customers / counterparties before any Copilot-generated content is shared externally?</t>
+          <t>Has a generative-AI model-governance review (NIST AI RMF 1.0 / ISO/IEC 42001, addressing the SR 26-2 / OCC 2026-13 generative-AI exclusion) been completed for Copilot?</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>AI disclosure template(s) reviewed by legal/compliance; Process documentation for applying disclosure to external content; SEC Marketing Rule alignment documentation; Evidence of disclosure usage in recent external communications</t>
+          <t>Generative-AI governance review document for Copilot; NIST AI RMF 1.0 alignment documentation; Bias testing and safety evaluation results; Responsible-AI principles adoption evidence</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr"/>
@@ -1114,12 +1114,12 @@
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>SEC Reg S-P -- Privacy of Consumer Financial Information</t>
+          <t>AI Disclosure, Transparency, and SEC Marketing Rule</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1139,12 +1139,12 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Have SEC Reg S-P / GLBA §501(b) privacy controls been reviewed for Copilot processing of customer NPI?</t>
+          <t>Is AI disclosure language presented to customers / counterparties before any Copilot-generated content is shared externally?</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Privacy impact assessment for Copilot NPI processing; DLP policy configuration preventing NPI surfacing outside authorized workflows; SEC Reg S-P alignment documentation for Copilot; GLBA §501(b) safeguards review covering Copilot</t>
+          <t>AI disclosure template(s) reviewed by legal/compliance; Process documentation for applying disclosure to external content; SEC Marketing Rule alignment documentation; Evidence of disclosure usage in recent external communications</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr"/>
@@ -1153,12 +1153,12 @@
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Record Keeping and Books-and-Records Compliance (SEC 17a-3/4, FINRA 4511)</t>
+          <t>SEC Reg S-P -- Privacy of Consumer Financial Information</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -1178,12 +1178,12 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Are Copilot interactions captured into the firm's books-and-records system per SEC Rule 17a-4 (where applicable)?</t>
+          <t>Have SEC Reg S-P / GLBA §501(b) privacy controls been reviewed for Copilot processing of customer NPI?</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Books-and-records policy covering Copilot interactions; WORM archive configuration for Copilot records (if applicable); Retrievability test results for examiner response readiness; Retention duration aligned to SEC 17a-4 / FINRA 4511</t>
+          <t>Privacy impact assessment for Copilot NPI processing; DLP policy configuration preventing NPI surfacing outside authorized workflows; SEC Reg S-P alignment documentation for Copilot; GLBA §501(b) safeguards review covering Copilot</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr"/>
@@ -1192,12 +1192,12 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>3.11</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Evidence Collection and Audit Attestation</t>
+          <t>Record Keeping and Books-and-Records Compliance (SEC 17a-3/4, FINRA 4511)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1217,12 +1217,12 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Is there a documented evidence-collection runbook used for Copilot-related audits and exam responses?</t>
+          <t>Are Copilot interactions captured into the firm's books-and-records system per SEC Rule 17a-4 (where applicable)?</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Evidence-collection runbook document with collector domain coverage; Sample evidence pack from most recent collection run; Audit attestation template aligned to regulatory requirements; Collection schedule and most recent run date</t>
+          <t>Books-and-records policy covering Copilot interactions; WORM archive configuration for Copilot records (if applicable); Retrievability test results for examiner response readiness; Retention duration aligned to SEC 17a-4 / FINRA 4511</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr"/>
@@ -1231,12 +1231,12 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>FFIEC IT Examination Handbook Alignment</t>
+          <t>Evidence Collection and Audit Attestation</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1256,25 +1256,181 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
+          <t>Is there a documented evidence-collection runbook used for Copilot-related audits and exam responses?</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
+          <t>Evidence-collection runbook document with collector domain coverage; Sample evidence pack from most recent collection run; Audit attestation template aligned to regulatory requirements; Collection schedule and most recent run date</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr"/>
       <c r="I22" s="7" t="inlineStr"/>
     </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>FFIEC IT Examination Handbook Alignment</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>P3 – Compliance &amp; Records</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr"/>
+      <c r="I23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Copilot Pages and Notebooks Retention and Provenance</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>P3 – Compliance &amp; Records</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Are branch-aware Copilot Pages, Notebook section-level coverage, and Loop component provenance addressed in retention and records-management policies?</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Retention policy covering Copilot Pages and Notebooks; Branch-aware retention configuration documentation; Provenance metadata strategy for Copilot-generated content; Section-level retention granularity documentation</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr"/>
+      <c r="I24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>4.15</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Copilot Cowork Governance</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Frontier preview enrollment record for tenant and admin accounts; Cowork availability configuration (scoped group or blocked) with approval; Approved Cowork plugin inventory and connector authentication records; Deployment/pinning approvals and supervision/audit coverage evidence</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr"/>
+      <c r="I25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Scout Governance</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr"/>
+      <c r="I26" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I22"/>
+  <autoFilter ref="A4:I26"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H22" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(controls): re-verify control 2.15 (Network Security) — update Last Verified to 2026-08-09
Re-verified technical claims: endpoints (M365 URLs and IP ranges), Microsoft 365 networking principles, Global Secure Access (Entra Internet Access & Private Access), Universal Tenant Restrictions, and Azure Private Link guidance. Regenerated content graph and checklist templates to keep mirrors consistent.

Sources:\n- https://learn.microsoft.com/en-us/microsoft-365/enterprise/microsoft-365-network-connectivity-principles\n- https://learn.microsoft.com/en-us/microsoft-365/enterprise/urls-and-ip-address-ranges\n- https://learn.microsoft.com/en-us/microsoft-365/enterprise/microsoft-365-networking-overview\n- https://learn.microsoft.com/en-us/entra/global-secure-access/overview-what-is-global-secure-access\n- https://learn.microsoft.com/en-us/entra/global-secure-access/how-to-universal-tenant-restrictions

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/compliance-officer-checklist.xlsx
+++ b/assessment/templates/compliance-officer-checklist.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>DLP Policies for Microsoft 365 Copilot Interactions</t>
+          <t>Are DLP policies for Copilot interactions configured, tested, and reviewed on a documented cadence?</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity Labels and Copilot Content Classification</t>
+          <t>Are sensitivity labels applied to Copilot-grounded content and label coverage reviewed on a documented cadence?</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>eDiscovery for Copilot-Generated Content</t>
+          <t>Are eDiscovery cases and holds configured to capture Copilot interaction content when legally required?</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">

</xml_diff>

<commit_message>
WIP(salvage): partial work from saul before timeout (issue #463)
Auto-committed by the timeout-salvage path so a long browser-driven conversion is not lost. Incomplete — a human should finish or discard.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/compliance-officer-checklist.xlsx
+++ b/assessment/templates/compliance-officer-checklist.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>DLP policy export showing 'Microsoft 365 Copilot and Copilot Chat' location or CopilotExperiences enforcement plane in scope; Three Copilot DLP scenarios present: sensitivity-label content processing, SIT prompt processing, and SIT external web-search restriction; Microsoft 365 admin center Web Content setting evidence showing web search scoped per approved user/group; Policy mode = Enforce (not Test / TestWithNotifications); Match-event report from Microsoft Purview portal &gt; Activity Explorer for the last 30 days; Override workflow document showing who can request and approve overrides</t>
+          <t>DLP policy export showing the 'Microsoft 365 Copilot and Copilot Chat' location and CopilotExperiences enforcement plane in scope; Applicable Copilot DLP scenarios present: sensitivity-label content processing, SIT prompt processing where available, SIT external web-search restriction, and assessment of preview external-email exclusion; Cloud Policy service evidence for Allow web search in Copilot showing the approved user/group scope; Policy mode and rollout evidence showing applicable rules are enforced after simulation; Match-event report from Microsoft Purview portal &gt; Solutions &gt; DSPM &gt; Discover &gt; Activity explorer for the last 30 days; Direct-upload file-content limitation test and compensating source-control evidence; Exception workflow showing who can request and approve policy-scope changes</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Privacy impact assessment for Copilot NPI processing; DLP policy configuration preventing NPI surfacing outside authorized workflows; SEC Reg S-P alignment documentation for Copilot; GLBA §501(b) safeguards review covering Copilot</t>
+          <t>Privacy impact assessment for Copilot NPI processing; Custom DLP policy configuration showing the Copilot location, applicable supported actions, mode, scope, and alerts; Synthetic tests for label exclusion, typed-prompt blocking where available, web-search restriction, external-email exclusion where available, and the direct-upload limitation; Purview Audit CopilotInteraction evidence and DSPM AI activity review; Copilot Pages and Notebooks SharePoint Embedded limitation review and admin-policy disposition; SEC Reg S-P alignment documentation for Copilot; GLBA §501(b) safeguards review covering Copilot</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr"/>

</xml_diff>